<commit_message>
Update analyses and tournament data
</commit_message>
<xml_diff>
--- a/tournament_data/all.xlsx
+++ b/tournament_data/all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Dropbox/passing_network/tournament_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA6297E-0FEE-0044-AF0B-EA3264AC0D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B99EAD5-9118-BD4D-B47A-7DC08479AA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="83">
   <si>
     <t>match_id</t>
   </si>
@@ -123,9 +123,6 @@
   </si>
   <si>
     <t>Sweden Women's</t>
-  </si>
-  <si>
-    <t>German Women's</t>
   </si>
   <si>
     <t>2025-07-13</t>
@@ -655,13 +652,13 @@
     <col min="3" max="4" width="18.1640625" customWidth="1"/>
     <col min="5" max="5" width="5.83203125" customWidth="1"/>
     <col min="6" max="6" width="7.6640625" customWidth="1"/>
-    <col min="7" max="7" width="7.5" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
     <col min="8" max="8" width="8" customWidth="1"/>
     <col min="9" max="9" width="7.33203125" customWidth="1"/>
     <col min="10" max="10" width="7" customWidth="1"/>
     <col min="11" max="11" width="7.83203125" customWidth="1"/>
     <col min="12" max="12" width="7.5" customWidth="1"/>
-    <col min="13" max="13" width="8.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.1640625" customWidth="1"/>
     <col min="14" max="14" width="8.5" customWidth="1"/>
     <col min="15" max="15" width="6" customWidth="1"/>
     <col min="16" max="16" width="7.33203125" customWidth="1"/>
@@ -682,43 +679,43 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>83</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>3</v>
@@ -757,40 +754,40 @@
         <v>14</v>
       </c>
       <c r="AC1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.2">
@@ -840,7 +837,7 @@
         <v>73</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q2">
         <v>0.92727272727272725</v>
@@ -894,7 +891,7 @@
         <v>2</v>
       </c>
       <c r="AH2">
-        <v>2441.2492772826758</v>
+        <v>2.4412492772826759</v>
       </c>
       <c r="AI2">
         <v>301</v>
@@ -920,10 +917,10 @@
         <v>4020846</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3">
         <v>0.35</v>
@@ -962,7 +959,7 @@
         <v>85</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q3">
         <v>0.81818181818181823</v>
@@ -992,7 +989,7 @@
         <v>8</v>
       </c>
       <c r="Z3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB3">
         <v>0.11031299999999999</v>
@@ -1013,7 +1010,7 @@
         <v>2</v>
       </c>
       <c r="AH3">
-        <v>2493.6750259708551</v>
+        <v>2.4936750259708553</v>
       </c>
       <c r="AI3">
         <v>525</v>
@@ -1025,7 +1022,7 @@
         <v>17</v>
       </c>
       <c r="AL3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN3">
         <v>8.0989000000000005E-2</v>
@@ -1036,10 +1033,10 @@
         <v>3998854</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4">
         <v>0.43</v>
@@ -1078,7 +1075,7 @@
         <v>86</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q4">
         <v>0.8</v>
@@ -1132,7 +1129,7 @@
         <v>2</v>
       </c>
       <c r="AH4">
-        <v>1737.8222256875999</v>
+        <v>1.7378222256875999</v>
       </c>
       <c r="AI4">
         <v>425</v>
@@ -1200,7 +1197,7 @@
         <v>78</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q5">
         <v>0.8</v>
@@ -1230,7 +1227,7 @@
         <v>14</v>
       </c>
       <c r="Z5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB5">
         <v>4.6346999999999999E-2</v>
@@ -1251,7 +1248,7 @@
         <v>2</v>
       </c>
       <c r="AH5">
-        <v>2247.475297372765</v>
+        <v>2.2474752973727652</v>
       </c>
       <c r="AI5">
         <v>441</v>
@@ -1263,7 +1260,7 @@
         <v>5</v>
       </c>
       <c r="AL5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN5">
         <v>0.20352000000000001</v>
@@ -1274,7 +1271,7 @@
         <v>3998855</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
         <v>26</v>
@@ -1316,7 +1313,7 @@
         <v>74</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q6">
         <v>0.89090909090909087</v>
@@ -1370,7 +1367,7 @@
         <v>2</v>
       </c>
       <c r="AH6">
-        <v>2118.5731006932469</v>
+        <v>2.1185731006932471</v>
       </c>
       <c r="AI6">
         <v>222</v>
@@ -1396,7 +1393,7 @@
         <v>3998840</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
@@ -1438,7 +1435,7 @@
         <v>60</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q7">
         <v>0.89090909090909087</v>
@@ -1492,7 +1489,7 @@
         <v>2</v>
       </c>
       <c r="AH7">
-        <v>1857.9461053888499</v>
+        <v>1.85794610538885</v>
       </c>
       <c r="AI7">
         <v>180</v>
@@ -1518,10 +1515,10 @@
         <v>3998855</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8">
         <v>0.26</v>
@@ -1560,7 +1557,7 @@
         <v>90</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q8">
         <v>0.79090909090909089</v>
@@ -1614,7 +1611,7 @@
         <v>2</v>
       </c>
       <c r="AH8">
-        <v>2414.2482523691451</v>
+        <v>2.4142482523691453</v>
       </c>
       <c r="AI8">
         <v>768</v>
@@ -1640,7 +1637,7 @@
         <v>3998847</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
         <v>26</v>
@@ -1682,7 +1679,7 @@
         <v>62</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q9">
         <v>0.89090909090909087</v>
@@ -1736,7 +1733,7 @@
         <v>3</v>
       </c>
       <c r="AH9">
-        <v>1970.126619688644</v>
+        <v>1.970126619688644</v>
       </c>
       <c r="AI9">
         <v>144</v>
@@ -1762,10 +1759,10 @@
         <v>3998854</v>
       </c>
       <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
         <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>35</v>
       </c>
       <c r="D10">
         <v>0.56999999999999995</v>
@@ -1804,7 +1801,7 @@
         <v>76</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q10">
         <v>0.89090909090909087</v>
@@ -1858,7 +1855,7 @@
         <v>2</v>
       </c>
       <c r="AH10">
-        <v>2009.5203277054659</v>
+        <v>2.0095203277054661</v>
       </c>
       <c r="AI10">
         <v>267</v>
@@ -1887,7 +1884,7 @@
         <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11">
         <v>0.46</v>
@@ -1926,7 +1923,7 @@
         <v>81</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q11">
         <v>0.88181818181818183</v>
@@ -1980,7 +1977,7 @@
         <v>2</v>
       </c>
       <c r="AH11">
-        <v>2002.7834508467729</v>
+        <v>2.0027834508467728</v>
       </c>
       <c r="AI11">
         <v>422</v>
@@ -2048,7 +2045,7 @@
         <v>71</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q12">
         <v>0.88181818181818183</v>
@@ -2102,7 +2099,7 @@
         <v>2</v>
       </c>
       <c r="AH12">
-        <v>1652.2251377329201</v>
+        <v>1.65222513773292</v>
       </c>
       <c r="AI12">
         <v>230</v>
@@ -2128,10 +2125,10 @@
         <v>3998858</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D13">
         <v>0.77</v>
@@ -2170,7 +2167,7 @@
         <v>65</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q13">
         <v>0.87272727272727268</v>
@@ -2224,7 +2221,7 @@
         <v>3</v>
       </c>
       <c r="AH13">
-        <v>1809.9638949028119</v>
+        <v>1.8099638949028118</v>
       </c>
       <c r="AI13">
         <v>234</v>
@@ -2250,7 +2247,7 @@
         <v>3998839</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
@@ -2292,7 +2289,7 @@
         <v>72</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q14">
         <v>0.87272727272727268</v>
@@ -2346,7 +2343,7 @@
         <v>2</v>
       </c>
       <c r="AH14">
-        <v>1474.198792349003</v>
+        <v>1.474198792349003</v>
       </c>
       <c r="AI14">
         <v>194</v>
@@ -2372,10 +2369,10 @@
         <v>3998859</v>
       </c>
       <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
         <v>31</v>
-      </c>
-      <c r="C15" t="s">
-        <v>32</v>
       </c>
       <c r="D15">
         <v>0.52</v>
@@ -2414,7 +2411,7 @@
         <v>76</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q15">
         <v>0.87272727272727268</v>
@@ -2468,7 +2465,7 @@
         <v>2</v>
       </c>
       <c r="AH15">
-        <v>2319.1278241658811</v>
+        <v>2.3191278241658813</v>
       </c>
       <c r="AI15">
         <v>285</v>
@@ -2494,10 +2491,10 @@
         <v>4018355</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D16">
         <v>0.6</v>
@@ -2536,7 +2533,7 @@
         <v>58</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q16">
         <v>0.87272727272727268</v>
@@ -2566,7 +2563,7 @@
         <v>13</v>
       </c>
       <c r="Z16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB16">
         <v>0.120356</v>
@@ -2587,7 +2584,7 @@
         <v>2</v>
       </c>
       <c r="AH16">
-        <v>2625.268238132956</v>
+        <v>2.6252682381329562</v>
       </c>
       <c r="AI16">
         <v>242</v>
@@ -2599,7 +2596,7 @@
         <v>7</v>
       </c>
       <c r="AL16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN16">
         <v>0.185832</v>
@@ -2610,10 +2607,10 @@
         <v>3998843</v>
       </c>
       <c r="B17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D17">
         <v>0.43</v>
@@ -2652,7 +2649,7 @@
         <v>82</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q17">
         <v>0.75454545454545452</v>
@@ -2706,7 +2703,7 @@
         <v>2</v>
       </c>
       <c r="AH17">
-        <v>2206.7475269739398</v>
+        <v>2.2067475269739396</v>
       </c>
       <c r="AI17">
         <v>410</v>
@@ -2732,10 +2729,10 @@
         <v>3998842</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18">
         <v>0.67</v>
@@ -2774,7 +2771,7 @@
         <v>67</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q18">
         <v>0.8545454545454545</v>
@@ -2828,7 +2825,7 @@
         <v>3</v>
       </c>
       <c r="AH18">
-        <v>1823.590506445094</v>
+        <v>1.8235905064450939</v>
       </c>
       <c r="AI18">
         <v>238</v>
@@ -2857,7 +2854,7 @@
         <v>20</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D19">
         <v>0.57999999999999996</v>
@@ -2896,7 +2893,7 @@
         <v>73</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q19">
         <v>0.8545454545454545</v>
@@ -2950,7 +2947,7 @@
         <v>2</v>
       </c>
       <c r="AH19">
-        <v>2350.167670581769</v>
+        <v>2.3501676705817691</v>
       </c>
       <c r="AI19">
         <v>318</v>
@@ -2976,10 +2973,10 @@
         <v>3998843</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D20">
         <v>0.56999999999999995</v>
@@ -3018,7 +3015,7 @@
         <v>77</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q20">
         <v>0.8545454545454545</v>
@@ -3072,7 +3069,7 @@
         <v>2</v>
       </c>
       <c r="AH20">
-        <v>2852.8399360051171</v>
+        <v>2.8528399360051173</v>
       </c>
       <c r="AI20">
         <v>356</v>
@@ -3140,7 +3137,7 @@
         <v>63</v>
       </c>
       <c r="P21" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q21">
         <v>0.8545454545454545</v>
@@ -3194,7 +3191,7 @@
         <v>3</v>
       </c>
       <c r="AH21">
-        <v>1966.460310819615</v>
+        <v>1.966460310819615</v>
       </c>
       <c r="AI21">
         <v>184</v>
@@ -3220,7 +3217,7 @@
         <v>4020077</v>
       </c>
       <c r="B22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22" t="s">
         <v>26</v>
@@ -3262,7 +3259,7 @@
         <v>72</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Q22">
         <v>0.84545454545454546</v>
@@ -3316,7 +3313,7 @@
         <v>2</v>
       </c>
       <c r="AH22">
-        <v>1814.9258607490301</v>
+        <v>1.8149258607490302</v>
       </c>
       <c r="AI22">
         <v>566</v>
@@ -3342,10 +3339,10 @@
         <v>3998836</v>
       </c>
       <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
         <v>44</v>
-      </c>
-      <c r="C23" t="s">
-        <v>45</v>
       </c>
       <c r="D23">
         <v>0.56000000000000005</v>
@@ -3384,7 +3381,7 @@
         <v>69</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q23">
         <v>0.74545454545454548</v>
@@ -3438,7 +3435,7 @@
         <v>2</v>
       </c>
       <c r="AH23">
-        <v>1749.999078933733</v>
+        <v>1.749999078933733</v>
       </c>
       <c r="AI23">
         <v>226</v>
@@ -3464,10 +3461,10 @@
         <v>3998850</v>
       </c>
       <c r="B24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D24">
         <v>0.25</v>
@@ -3506,7 +3503,7 @@
         <v>89</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q24">
         <v>0.74545454545454548</v>
@@ -3560,7 +3557,7 @@
         <v>2</v>
       </c>
       <c r="AH24">
-        <v>2583.1919763610881</v>
+        <v>2.5831919763610882</v>
       </c>
       <c r="AI24">
         <v>578</v>
@@ -3586,7 +3583,7 @@
         <v>4018357</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" t="s">
         <v>23</v>
@@ -3628,7 +3625,7 @@
         <v>85</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q25">
         <v>0.62222222222222223</v>
@@ -3658,7 +3655,7 @@
         <v>6</v>
       </c>
       <c r="Z25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB25">
         <v>0.18415000000000001</v>
@@ -3679,7 +3676,7 @@
         <v>2</v>
       </c>
       <c r="AH25">
-        <v>2337.9596171785302</v>
+        <v>2.3379596171785302</v>
       </c>
       <c r="AI25">
         <v>456</v>
@@ -3691,7 +3688,7 @@
         <v>11</v>
       </c>
       <c r="AL25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN25">
         <v>0.142152</v>
@@ -3705,7 +3702,7 @@
         <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D26">
         <v>0.52</v>
@@ -3744,7 +3741,7 @@
         <v>79</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q26">
         <v>0.83636363636363631</v>
@@ -3774,7 +3771,7 @@
         <v>5</v>
       </c>
       <c r="Z26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB26">
         <v>0.20352000000000001</v>
@@ -3795,7 +3792,7 @@
         <v>2</v>
       </c>
       <c r="AH26">
-        <v>2143.3467986018281</v>
+        <v>2.143346798601828</v>
       </c>
       <c r="AI26">
         <v>352</v>
@@ -3807,7 +3804,7 @@
         <v>14</v>
       </c>
       <c r="AL26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN26">
         <v>4.6346999999999999E-2</v>
@@ -3821,7 +3818,7 @@
         <v>28</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D27">
         <v>0.51</v>
@@ -3860,7 +3857,7 @@
         <v>82</v>
       </c>
       <c r="P27" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q27">
         <v>0.83636363636363631</v>
@@ -3914,7 +3911,7 @@
         <v>2</v>
       </c>
       <c r="AH27">
-        <v>2587.1018560606062</v>
+        <v>2.5871018560606061</v>
       </c>
       <c r="AI27">
         <v>338</v>
@@ -3943,7 +3940,7 @@
         <v>28</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D28">
         <v>0.54</v>
@@ -3982,7 +3979,7 @@
         <v>77</v>
       </c>
       <c r="P28" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q28">
         <v>0.82727272727272727</v>
@@ -4036,7 +4033,7 @@
         <v>2</v>
       </c>
       <c r="AH28">
-        <v>1199.326638156969</v>
+        <v>1.1993266381569689</v>
       </c>
       <c r="AI28">
         <v>365</v>
@@ -4062,10 +4059,10 @@
         <v>3998850</v>
       </c>
       <c r="B29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D29">
         <v>0.75</v>
@@ -4104,7 +4101,7 @@
         <v>64</v>
       </c>
       <c r="P29" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q29">
         <v>0.82727272727272727</v>
@@ -4158,7 +4155,7 @@
         <v>2</v>
       </c>
       <c r="AH29">
-        <v>1346.1246593153389</v>
+        <v>1.3461246593153389</v>
       </c>
       <c r="AI29">
         <v>212</v>
@@ -4226,7 +4223,7 @@
         <v>71</v>
       </c>
       <c r="P30" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q30">
         <v>0.72727272727272729</v>
@@ -4280,7 +4277,7 @@
         <v>2</v>
       </c>
       <c r="AH30">
-        <v>1699.3926926173319</v>
+        <v>1.6993926926173319</v>
       </c>
       <c r="AI30">
         <v>295</v>
@@ -4306,10 +4303,10 @@
         <v>3998851</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D31">
         <v>0.52</v>
@@ -4348,7 +4345,7 @@
         <v>77</v>
       </c>
       <c r="P31" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q31">
         <v>0.82727272727272727</v>
@@ -4402,7 +4399,7 @@
         <v>2</v>
       </c>
       <c r="AH31">
-        <v>1583.9478053370251</v>
+        <v>1.5839478053370251</v>
       </c>
       <c r="AI31">
         <v>308</v>
@@ -4470,7 +4467,7 @@
         <v>70</v>
       </c>
       <c r="P32" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q32">
         <v>0.81818181818181823</v>
@@ -4524,7 +4521,7 @@
         <v>2</v>
       </c>
       <c r="AH32">
-        <v>2203.1158600623162</v>
+        <v>2.203115860062316</v>
       </c>
       <c r="AI32">
         <v>240</v>
@@ -4592,7 +4589,7 @@
         <v>73</v>
       </c>
       <c r="P33" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q33">
         <v>0.81818181818181823</v>
@@ -4646,7 +4643,7 @@
         <v>3</v>
       </c>
       <c r="AH33">
-        <v>1982.540222053872</v>
+        <v>1.9825402220538719</v>
       </c>
       <c r="AI33">
         <v>337</v>
@@ -4672,10 +4669,10 @@
         <v>4018354</v>
       </c>
       <c r="B34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D34">
         <v>0.51</v>
@@ -4714,7 +4711,7 @@
         <v>77</v>
       </c>
       <c r="P34" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q34">
         <v>0.81818181818181823</v>
@@ -4768,7 +4765,7 @@
         <v>2</v>
       </c>
       <c r="AH34">
-        <v>2130.1582388977008</v>
+        <v>2.130158238897701</v>
       </c>
       <c r="AI34">
         <v>368</v>
@@ -4794,10 +4791,10 @@
         <v>4018357</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D35">
         <v>0.74</v>
@@ -4836,7 +4833,7 @@
         <v>51</v>
       </c>
       <c r="P35" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q35">
         <v>0.80909090909090908</v>
@@ -4866,7 +4863,7 @@
         <v>11</v>
       </c>
       <c r="Z35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB35">
         <v>0.142152</v>
@@ -4887,7 +4884,7 @@
         <v>2</v>
       </c>
       <c r="AH35">
-        <v>1688.855529252997</v>
+        <v>1.688855529252997</v>
       </c>
       <c r="AI35">
         <v>122</v>
@@ -4899,7 +4896,7 @@
         <v>6</v>
       </c>
       <c r="AL35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN35">
         <v>0.18415000000000001</v>
@@ -4910,7 +4907,7 @@
         <v>4020846</v>
       </c>
       <c r="B36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C36" t="s">
         <v>26</v>
@@ -4952,7 +4949,7 @@
         <v>74</v>
       </c>
       <c r="P36" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q36">
         <v>0.80909090909090908</v>
@@ -4982,7 +4979,7 @@
         <v>17</v>
       </c>
       <c r="Z36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB36">
         <v>8.0989000000000005E-2</v>
@@ -5003,7 +5000,7 @@
         <v>2</v>
       </c>
       <c r="AH36">
-        <v>2322.5724357914842</v>
+        <v>2.3225724357914843</v>
       </c>
       <c r="AI36">
         <v>336</v>
@@ -5015,7 +5012,7 @@
         <v>8</v>
       </c>
       <c r="AL36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN36">
         <v>0.11031299999999999</v>
@@ -5026,10 +5023,10 @@
         <v>3998846</v>
       </c>
       <c r="B37" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D37">
         <v>0.56999999999999995</v>
@@ -5068,7 +5065,7 @@
         <v>75</v>
       </c>
       <c r="P37" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q37">
         <v>0.80303030303030298</v>
@@ -5098,7 +5095,7 @@
         <v>4</v>
       </c>
       <c r="Z37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB37">
         <v>5.3744E-2</v>
@@ -5119,7 +5116,7 @@
         <v>2</v>
       </c>
       <c r="AH37">
-        <v>2587.748500605881</v>
+        <v>2.5877485006058811</v>
       </c>
       <c r="AI37">
         <v>276</v>
@@ -5131,7 +5128,7 @@
         <v>10</v>
       </c>
       <c r="AL37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN37">
         <v>7.3607000000000006E-2</v>
@@ -5142,7 +5139,7 @@
         <v>4018354</v>
       </c>
       <c r="B38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C38" t="s">
         <v>18</v>
@@ -5184,7 +5181,7 @@
         <v>78</v>
       </c>
       <c r="P38" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q38">
         <v>0.79090909090909089</v>
@@ -5238,7 +5235,7 @@
         <v>2</v>
       </c>
       <c r="AH38">
-        <v>2091.3919467949709</v>
+        <v>2.0913919467949706</v>
       </c>
       <c r="AI38">
         <v>390</v>
@@ -5264,7 +5261,7 @@
         <v>3998836</v>
       </c>
       <c r="B39" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C39" t="s">
         <v>21</v>
@@ -5306,7 +5303,7 @@
         <v>78</v>
       </c>
       <c r="P39" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q39">
         <v>0.69090909090909092</v>
@@ -5360,7 +5357,7 @@
         <v>2</v>
       </c>
       <c r="AH39">
-        <v>2334.4049774154591</v>
+        <v>2.3344049774154589</v>
       </c>
       <c r="AI39">
         <v>354</v>
@@ -5386,7 +5383,7 @@
         <v>4018355</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C40" t="s">
         <v>29</v>
@@ -5428,7 +5425,7 @@
         <v>74</v>
       </c>
       <c r="P40" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q40">
         <v>0.69090909090909092</v>
@@ -5458,7 +5455,7 @@
         <v>7</v>
       </c>
       <c r="Z40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB40">
         <v>0.185832</v>
@@ -5479,7 +5476,7 @@
         <v>2</v>
       </c>
       <c r="AH40">
-        <v>2093.306242079962</v>
+        <v>2.093306242079962</v>
       </c>
       <c r="AI40">
         <v>468</v>
@@ -5491,7 +5488,7 @@
         <v>13</v>
       </c>
       <c r="AL40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN40">
         <v>0.120356</v>
@@ -5502,10 +5499,10 @@
         <v>3998851</v>
       </c>
       <c r="B41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D41">
         <v>0.48</v>
@@ -5544,7 +5541,7 @@
         <v>79</v>
       </c>
       <c r="P41" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q41">
         <v>0.79090909090909089</v>
@@ -5598,7 +5595,7 @@
         <v>2</v>
       </c>
       <c r="AH41">
-        <v>2262.027441045936</v>
+        <v>2.262027441045936</v>
       </c>
       <c r="AI41">
         <v>373</v>
@@ -5624,10 +5621,10 @@
         <v>3998847</v>
       </c>
       <c r="B42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C42" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D42">
         <v>0.2</v>
@@ -5666,7 +5663,7 @@
         <v>89</v>
       </c>
       <c r="P42" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q42">
         <v>0.58181818181818179</v>
@@ -5720,7 +5717,7 @@
         <v>2</v>
       </c>
       <c r="AH42">
-        <v>2193.9799070365161</v>
+        <v>2.1939799070365162</v>
       </c>
       <c r="AI42">
         <v>717</v>
@@ -5746,10 +5743,10 @@
         <v>3998841</v>
       </c>
       <c r="B43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D43">
         <v>0.42</v>
@@ -5788,7 +5785,7 @@
         <v>74</v>
       </c>
       <c r="P43" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q43">
         <v>0.68181818181818177</v>
@@ -5842,7 +5839,7 @@
         <v>2</v>
       </c>
       <c r="AH43">
-        <v>2502.389635041156</v>
+        <v>2.5023896350411561</v>
       </c>
       <c r="AI43">
         <v>331</v>
@@ -5910,7 +5907,7 @@
         <v>88</v>
       </c>
       <c r="P44" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q44">
         <v>0.78181818181818186</v>
@@ -5964,7 +5961,7 @@
         <v>2</v>
       </c>
       <c r="AH44">
-        <v>2134.1234356666059</v>
+        <v>2.1341234356666061</v>
       </c>
       <c r="AI44">
         <v>616</v>
@@ -5990,10 +5987,10 @@
         <v>3998838</v>
       </c>
       <c r="B45" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45" t="s">
         <v>37</v>
-      </c>
-      <c r="C45" t="s">
-        <v>38</v>
       </c>
       <c r="D45">
         <v>0.47</v>
@@ -6032,7 +6029,7 @@
         <v>82</v>
       </c>
       <c r="P45" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q45">
         <v>0.78181818181818186</v>
@@ -6086,7 +6083,7 @@
         <v>2</v>
       </c>
       <c r="AH45">
-        <v>2807.4579443780849</v>
+        <v>2.8074579443780849</v>
       </c>
       <c r="AI45">
         <v>327</v>
@@ -6154,7 +6151,7 @@
         <v>81</v>
       </c>
       <c r="P46" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q46">
         <v>0.77272727272727271</v>
@@ -6208,7 +6205,7 @@
         <v>2</v>
       </c>
       <c r="AH46">
-        <v>2018.511459194641</v>
+        <v>2.0185114591946411</v>
       </c>
       <c r="AI46">
         <v>524</v>
@@ -6234,10 +6231,10 @@
         <v>3998838</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C47" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D47">
         <v>0.53</v>
@@ -6276,7 +6273,7 @@
         <v>80</v>
       </c>
       <c r="P47" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q47">
         <v>0.77272727272727271</v>
@@ -6330,7 +6327,7 @@
         <v>2</v>
       </c>
       <c r="AH47">
-        <v>2437.802382876383</v>
+        <v>2.4378023828763831</v>
       </c>
       <c r="AI47">
         <v>302</v>
@@ -6356,10 +6353,10 @@
         <v>3998859</v>
       </c>
       <c r="B48" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C48" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D48">
         <v>0.48</v>
@@ -6398,7 +6395,7 @@
         <v>76</v>
       </c>
       <c r="P48" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q48">
         <v>0.77272727272727271</v>
@@ -6452,7 +6449,7 @@
         <v>2</v>
       </c>
       <c r="AH48">
-        <v>1901.526211749527</v>
+        <v>1.9015262117495271</v>
       </c>
       <c r="AI48">
         <v>296</v>
@@ -6520,7 +6517,7 @@
         <v>82</v>
       </c>
       <c r="P49" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q49">
         <v>0.77272727272727271</v>
@@ -6574,7 +6571,7 @@
         <v>2</v>
       </c>
       <c r="AH49">
-        <v>2419.8155242195089</v>
+        <v>2.419815524219509</v>
       </c>
       <c r="AI49">
         <v>411</v>
@@ -6600,10 +6597,10 @@
         <v>4020005</v>
       </c>
       <c r="B50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C50" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D50">
         <v>0.57999999999999996</v>
@@ -6642,7 +6639,7 @@
         <v>76</v>
       </c>
       <c r="P50" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Q50">
         <v>0.87272727272727268</v>
@@ -6696,7 +6693,7 @@
         <v>2</v>
       </c>
       <c r="AH50">
-        <v>2400.8540296518959</v>
+        <v>2.4008540296518959</v>
       </c>
       <c r="AI50">
         <v>283</v>
@@ -6722,10 +6719,10 @@
         <v>3998842</v>
       </c>
       <c r="B51" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C51" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D51">
         <v>0.33</v>
@@ -6764,7 +6761,7 @@
         <v>87</v>
       </c>
       <c r="P51" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q51">
         <v>0.77272727272727271</v>
@@ -6818,7 +6815,7 @@
         <v>2</v>
       </c>
       <c r="AH51">
-        <v>1916.65514072061</v>
+        <v>1.9166551407206101</v>
       </c>
       <c r="AI51">
         <v>509</v>
@@ -6844,10 +6841,10 @@
         <v>3998840</v>
       </c>
       <c r="B52" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C52" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D52">
         <v>0.3</v>
@@ -6886,7 +6883,7 @@
         <v>87</v>
       </c>
       <c r="P52" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q52">
         <v>0.58333333333333337</v>
@@ -6940,7 +6937,7 @@
         <v>2</v>
       </c>
       <c r="AH52">
-        <v>2138.6413560556871</v>
+        <v>2.1386413560556869</v>
       </c>
       <c r="AI52">
         <v>559</v>
@@ -6966,7 +6963,7 @@
         <v>4020077</v>
       </c>
       <c r="B53" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C53" t="s">
         <v>23</v>
@@ -7008,7 +7005,7 @@
         <v>87</v>
       </c>
       <c r="P53" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Q53">
         <v>0.66363636363636369</v>
@@ -7062,7 +7059,7 @@
         <v>2</v>
       </c>
       <c r="AH53">
-        <v>1832.841582750154</v>
+        <v>1.8328415827501541</v>
       </c>
       <c r="AI53">
         <v>194</v>
@@ -7130,7 +7127,7 @@
         <v>86</v>
       </c>
       <c r="P54" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q54">
         <v>0.66363636363636369</v>
@@ -7184,7 +7181,7 @@
         <v>2</v>
       </c>
       <c r="AH54">
-        <v>2140.8171787173192</v>
+        <v>2.1408171787173194</v>
       </c>
       <c r="AI54">
         <v>489</v>
@@ -7252,7 +7249,7 @@
         <v>79</v>
       </c>
       <c r="P55" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q55">
         <v>0.75454545454545452</v>
@@ -7306,7 +7303,7 @@
         <v>2</v>
       </c>
       <c r="AH55">
-        <v>1758.207545986178</v>
+        <v>1.7582075459861781</v>
       </c>
       <c r="AI55">
         <v>334</v>
@@ -7332,7 +7329,7 @@
         <v>3998841</v>
       </c>
       <c r="B56" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C56" t="s">
         <v>29</v>
@@ -7374,7 +7371,7 @@
         <v>66</v>
       </c>
       <c r="P56" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q56">
         <v>0.75454545454545452</v>
@@ -7428,7 +7425,7 @@
         <v>2</v>
       </c>
       <c r="AH56">
-        <v>1890.2365130291</v>
+        <v>1.8902365130291001</v>
       </c>
       <c r="AI56">
         <v>233</v>
@@ -7496,7 +7493,7 @@
         <v>85</v>
       </c>
       <c r="P57" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q57">
         <v>0.75454545454545452</v>
@@ -7550,7 +7547,7 @@
         <v>2</v>
       </c>
       <c r="AH57">
-        <v>2244.7271037221599</v>
+        <v>2.2447271037221599</v>
       </c>
       <c r="AI57">
         <v>516</v>
@@ -7576,10 +7573,10 @@
         <v>3998846</v>
       </c>
       <c r="B58" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C58" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D58">
         <v>0.43</v>
@@ -7618,7 +7615,7 @@
         <v>80</v>
       </c>
       <c r="P58" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q58">
         <v>0.75454545454545452</v>
@@ -7648,7 +7645,7 @@
         <v>10</v>
       </c>
       <c r="Z58" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AB58">
         <v>7.3607000000000006E-2</v>
@@ -7669,7 +7666,7 @@
         <v>2</v>
       </c>
       <c r="AH58">
-        <v>2335.9743311835568</v>
+        <v>2.3359743311835568</v>
       </c>
       <c r="AI58">
         <v>364</v>
@@ -7681,7 +7678,7 @@
         <v>4</v>
       </c>
       <c r="AL58" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AN58">
         <v>5.3744E-2</v>
@@ -7695,7 +7692,7 @@
         <v>22</v>
       </c>
       <c r="C59" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D59">
         <v>0.46</v>
@@ -7734,7 +7731,7 @@
         <v>76</v>
       </c>
       <c r="P59" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q59">
         <v>0.74545454545454548</v>
@@ -7788,7 +7785,7 @@
         <v>3</v>
       </c>
       <c r="AH59">
-        <v>2605.5793736214318</v>
+        <v>2.6055793736214317</v>
       </c>
       <c r="AI59">
         <v>341</v>
@@ -7856,7 +7853,7 @@
         <v>75</v>
       </c>
       <c r="P60" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q60">
         <v>0.73636363636363633</v>
@@ -7910,7 +7907,7 @@
         <v>2</v>
       </c>
       <c r="AH60">
-        <v>2353.6328647227392</v>
+        <v>2.3536328647227394</v>
       </c>
       <c r="AI60">
         <v>317</v>
@@ -7936,10 +7933,10 @@
         <v>4020005</v>
       </c>
       <c r="B61" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C61" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D61">
         <v>0.42</v>
@@ -7978,7 +7975,7 @@
         <v>83</v>
       </c>
       <c r="P61" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Q61">
         <v>0.72727272727272729</v>
@@ -8032,7 +8029,7 @@
         <v>2</v>
       </c>
       <c r="AH61">
-        <v>2240.1168869234498</v>
+        <v>2.2401168869234498</v>
       </c>
       <c r="AI61">
         <v>412</v>
@@ -8058,10 +8055,10 @@
         <v>3998839</v>
       </c>
       <c r="B62" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C62" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D62">
         <v>0.28999999999999998</v>
@@ -8100,7 +8097,7 @@
         <v>88</v>
       </c>
       <c r="P62" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q62">
         <v>0.70909090909090911</v>
@@ -8154,7 +8151,7 @@
         <v>2</v>
       </c>
       <c r="AH62">
-        <v>1985.26300167827</v>
+        <v>1.98526300167827</v>
       </c>
       <c r="AI62">
         <v>610</v>
@@ -8180,10 +8177,10 @@
         <v>3998858</v>
       </c>
       <c r="B63" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C63" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D63">
         <v>0.23</v>
@@ -8222,7 +8219,7 @@
         <v>91</v>
       </c>
       <c r="P63" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Q63">
         <v>0.7</v>
@@ -8276,7 +8273,7 @@
         <v>2</v>
       </c>
       <c r="AH63">
-        <v>2252.6232705712032</v>
+        <v>2.252623270571203</v>
       </c>
       <c r="AI63">
         <v>747</v>

</xml_diff>